<commit_message>
Mescla arquivos do projeto JamesSinc
</commit_message>
<xml_diff>
--- a/uploads/ELETROPEL_2.xlsx
+++ b/uploads/ELETROPEL_2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\james.santos\Documents\28-07\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E889C67-3626-4699-AC1C-64B83E774B13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1D0D4CC-3FBA-405C-ABCE-026D0BDED6E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{578B0778-6105-4924-AD08-9FFA4E9E5CEE}"/>
   </bookViews>
@@ -314,6 +314,9 @@
     <t>QTD</t>
   </si>
   <si>
+    <t>VALOR</t>
+  </si>
+  <si>
     <t>Descrição LBDIESEL</t>
   </si>
   <si>
@@ -381,9 +384,6 @@
   </si>
   <si>
     <t>PREÇO</t>
-  </si>
-  <si>
-    <t>MARCA</t>
   </si>
 </sst>
 </file>
@@ -800,10 +800,10 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>89</v>
@@ -815,7 +815,7 @@
         <v>90</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>113</v>
+        <v>91</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>114</v>
@@ -841,7 +841,7 @@
         <v>27.45</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -864,7 +864,7 @@
         <v>17.48</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -910,7 +910,7 @@
         <v>32.99</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -933,7 +933,7 @@
         <v>11.45</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -1002,7 +1002,7 @@
         <v>0.41</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -1048,7 +1048,7 @@
         <v>5.55</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -1094,7 +1094,7 @@
         <v>112.55</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -1117,7 +1117,7 @@
         <v>11.15</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
@@ -1140,7 +1140,7 @@
         <v>27.8</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
@@ -1186,7 +1186,7 @@
         <v>139.9</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
@@ -1232,7 +1232,7 @@
         <v>281.14999999999998</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
@@ -1278,7 +1278,7 @@
         <v>131</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
@@ -1298,7 +1298,7 @@
         <v>1</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G22" s="1"/>
     </row>
@@ -1391,7 +1391,7 @@
         <v>21</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
@@ -1411,7 +1411,7 @@
         <v>1</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G27" s="1"/>
     </row>
@@ -1458,7 +1458,7 @@
         <v>21.35</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
@@ -1478,7 +1478,7 @@
         <v>2</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G30" s="1"/>
     </row>
@@ -1525,7 +1525,7 @@
         <v>58.15</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
@@ -1571,7 +1571,7 @@
         <v>93.6</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
@@ -1594,7 +1594,7 @@
         <v>18.149999999999999</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
@@ -1617,7 +1617,7 @@
         <v>33.9</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
@@ -1663,7 +1663,7 @@
         <v>7.75</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
@@ -1683,7 +1683,7 @@
         <v>3</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G39" s="1"/>
     </row>
@@ -1704,7 +1704,7 @@
         <v>1</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G40" s="1"/>
     </row>
@@ -1751,7 +1751,7 @@
         <v>17.5</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
@@ -1774,7 +1774,7 @@
         <v>27.15</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
@@ -1794,7 +1794,7 @@
         <v>4</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G44" s="1"/>
     </row>
@@ -1818,7 +1818,7 @@
         <v>1571</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
@@ -2140,7 +2140,7 @@
         <v>29.8</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">
@@ -2209,7 +2209,7 @@
         <v>30.5</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.3">
@@ -2229,7 +2229,7 @@
         <v>5</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G63" s="1"/>
     </row>
@@ -2342,7 +2342,7 @@
         <v>6</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G68" s="1"/>
     </row>
@@ -2389,7 +2389,7 @@
         <v>50.35</v>
       </c>
       <c r="G70" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.3">
@@ -2435,7 +2435,7 @@
         <v>20.9</v>
       </c>
       <c r="G72" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
@@ -2458,7 +2458,7 @@
         <v>4.78</v>
       </c>
       <c r="G73" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
@@ -2481,7 +2481,7 @@
         <v>63.65</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.3">
@@ -2619,7 +2619,7 @@
         <v>98.55</v>
       </c>
       <c r="G80" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.3">
@@ -2642,7 +2642,7 @@
         <v>9.8000000000000007</v>
       </c>
       <c r="G81" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>